<commit_message>
Geração e validação de respostas
</commit_message>
<xml_diff>
--- a/Tyche_Pay_Mapeamento_de_Documentos.xlsx
+++ b/Tyche_Pay_Mapeamento_de_Documentos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\joaom\OneDrive\Documentos\Challenge-AgenteIA-da-alura\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FCEE789-564E-41C8-A600-855829291BDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CF97D1A-58D2-4904-8730-2FDE103ECF5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,14 +17,14 @@
     <sheet name="Legenda e Processo" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Mapeamento de Documentos'!$A$1:$L$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Mapeamento de Documentos'!$A$1:$L$19</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="156">
   <si>
     <t>Nome do Documento</t>
   </si>
@@ -83,9 +83,6 @@
     <t>1.0</t>
   </si>
   <si>
-    <t>Ago/2026</t>
-  </si>
-  <si>
     <t>Revisado</t>
   </si>
   <si>
@@ -182,9 +179,6 @@
     <t>Reuniões / Governança Corporativa</t>
   </si>
   <si>
-    <t>01/08/2026</t>
-  </si>
-  <si>
     <t>Interno (uso corporativo)</t>
   </si>
   <si>
@@ -479,26 +473,55 @@
     <t>Qualidade</t>
   </si>
   <si>
-    <t>Auditoria Interna / SLA de Atendimento</t>
-  </si>
-  <si>
     <t>Q2 2026</t>
   </si>
   <si>
-    <t>Q2 2026 (ago/2026 — data de emissão do relatório)</t>
-  </si>
-  <si>
     <t>Complementa o Playbook e o FAQ com métricas quantitativas de qualidade (NPS, FCR, TME, TMA); contém plano de ação com recomendações (ex.: treinamento de reciclagem LGPD) que pode virar gatilho de atualização de outros documentos — vale revisar trimestralmente junto com a próxima auditoria.</t>
   </si>
   <si>
     <t>Tyche Pay - Relatório de Auditoria Interna e SLA de Atendimento.pdf</t>
+  </si>
+  <si>
+    <t>Diretório de Contatos Internos e Responsáveis por Área</t>
+  </si>
+  <si>
+    <t>Diretório Organizacional / Canais de Contato</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Contém dados pessoais de colaboradores (nome, e-mail direto, ramal individual) misturados a canais institucionais genéricos (0800, e-mails de departamento). Manter estritamente interno — não incluir em qualquer versão do agente com acesso externo/client-facing. Revela que </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Juliana Martins é a Head de RH</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>: atualizar o owner do Manual de Onboarding e da Política de Benefícios de "a definir" para "Juliana Martins (Head de RH)".</t>
+    </r>
+  </si>
+  <si>
+    <t>Tyche Pay - Diretório de Contatos Internos e Responsáveis por Área.pdf</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -544,6 +567,14 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -598,7 +629,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -618,10 +649,13 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -926,7 +960,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33.88671875" bestFit="1" customWidth="1"/>
@@ -981,7 +1015,7 @@
         <v>11</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
@@ -1006,199 +1040,199 @@
       <c r="G2" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="11">
+        <v>46235</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="L2" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="L2" s="2" t="s">
-        <v>23</v>
-      </c>
       <c r="M2" s="6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>26</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>27</v>
       </c>
       <c r="G3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="11">
+        <v>46235</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="J3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L3" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="K3" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="M3" s="6" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>32</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>33</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="11">
+        <v>46235</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="J4" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M4" s="6" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>37</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="11">
+        <v>46235</v>
+      </c>
+      <c r="I5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I5" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="J5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="K5" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="L5" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="L5" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="M5" s="6" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="11">
+        <v>46235</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L6" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="H6" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="K6" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>46</v>
-      </c>
       <c r="M6" s="6" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>48</v>
-      </c>
       <c r="D7" s="2" t="s">
         <v>16</v>
       </c>
@@ -1206,39 +1240,39 @@
         <v>16</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="11">
+        <v>46235</v>
+      </c>
+      <c r="I7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I7" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="J7" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>51</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>16</v>
@@ -1252,157 +1286,157 @@
       <c r="G8" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="11">
+        <v>46235</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L8" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="I8" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="K8" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>54</v>
-      </c>
       <c r="M8" s="6" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F9" s="2" t="s">
+      <c r="H9" s="11">
+        <v>46235</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J9" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="K9" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L9" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="K9" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>60</v>
-      </c>
       <c r="M9" s="6" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="D10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>64</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="11">
+        <v>46235</v>
+      </c>
+      <c r="I10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I10" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="J10" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="L10" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="K10" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="L10" s="2" t="s">
-        <v>67</v>
-      </c>
       <c r="M10" s="6" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="C11" s="2" t="s">
+      <c r="H11" s="11">
+        <v>46236</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J11" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="D11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="G11" s="2" t="s">
+      <c r="K11" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="H11" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I11" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J11" s="2" t="s">
+      <c r="L11" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="K11" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="L11" s="2" t="s">
-        <v>73</v>
-      </c>
       <c r="M11" s="6" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>16</v>
@@ -1411,39 +1445,39 @@
         <v>16</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="H12" s="11">
+        <v>46235</v>
+      </c>
+      <c r="I12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I12" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="J12" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="L12" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="K12" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>78</v>
-      </c>
       <c r="M12" s="6" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>16</v>
@@ -1452,237 +1486,278 @@
         <v>16</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="H13" s="11">
+        <v>46235</v>
+      </c>
+      <c r="I13" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I13" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="J13" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="M13" s="6" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="B14" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C14" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="F14" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="H14" s="11">
+        <v>46235</v>
+      </c>
+      <c r="I14" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="G14" s="2" t="s">
+      <c r="J14" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="H14" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="I14" s="2" t="s">
+      <c r="K14" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="J14" s="2" t="s">
+      <c r="L14" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="K14" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>90</v>
-      </c>
       <c r="M14" s="6" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>93</v>
       </c>
       <c r="G15" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="H15" s="11">
+        <v>46235</v>
+      </c>
+      <c r="I15" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I15" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="J15" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M15" s="6" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="D16" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F16" s="2" t="s">
-        <v>97</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="H16" s="11">
+        <v>46235</v>
+      </c>
+      <c r="I16" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I16" s="2" t="s">
-        <v>20</v>
-      </c>
       <c r="J16" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="M16" s="6" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>95</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E17" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F17" s="2" t="s">
-        <v>97</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H17" s="2" t="s">
+      <c r="H17" s="11">
+        <v>46235</v>
+      </c>
+      <c r="I17" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="I17" s="6" t="s">
-        <v>20</v>
-      </c>
       <c r="J17" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M17" s="6" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="105.6" x14ac:dyDescent="0.3">
+      <c r="A18" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" ht="105.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="10" t="s">
+      <c r="C18" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="H18" s="11">
+        <v>46239</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="K18" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L18" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="M18" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="D18" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="G18" s="2" t="s">
+    </row>
+    <row r="19" spans="1:13" ht="136.80000000000001" x14ac:dyDescent="0.3">
+      <c r="A19" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="H18" s="6" t="s">
+      <c r="B19" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="I18" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="J18" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="K18" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="L18" s="2" t="s">
+      <c r="D19" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H19" s="11">
+        <v>46235</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="K19" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L19" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="M18" s="6" t="s">
+      <c r="M19" s="6" t="s">
         <v>155</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L17" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:L19" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1697,159 +1772,159 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="B1" s="8"/>
+      <c r="A1" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="B1" s="9"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="B3" s="8"/>
+      <c r="A3" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="B3" s="9"/>
     </row>
     <row r="4" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
         <v>109</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="B9" s="8"/>
+      <c r="B9" s="9"/>
     </row>
     <row r="10" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="B13" s="4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="B15" s="8"/>
+      <c r="B15" s="9"/>
     </row>
     <row r="16" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="B20" s="8"/>
+      <c r="A20" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="B20" s="9"/>
     </row>
     <row r="21" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="B22" s="4" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="B24" s="8"/>
+      <c r="B24" s="9"/>
     </row>
     <row r="25" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>